<commit_message>
Improve VBA config builder workflow
</commit_message>
<xml_diff>
--- a/config/templates/config_builder_template.xlsx
+++ b/config/templates/config_builder_template.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="R80dd547012784d5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Setup" sheetId="2" r:id="Rc93f1369248f41c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="3" r:id="Re7cf8ae88ae14f5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Sources" sheetId="4" r:id="R1dc519c632044114"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Args" sheetId="5" r:id="Re7ba7b8898784901"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sector Defaults" sheetId="6" r:id="R80745a5c3eed41fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Defaults" sheetId="7" r:id="Rb5011eee0aa444f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Control" sheetId="8" r:id="Re810ee0ef4ad4c01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="9" r:id="R4cae15a0bd664528"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="10" r:id="R2943e3555eb84ff8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="R199d44105a7b4e45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Setup" sheetId="2" r:id="R1dff62dee720488c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="3" r:id="R1c7878bb832d4471"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Sources" sheetId="4" r:id="Rd88ffaeb220e4cdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Args" sheetId="5" r:id="R1ec4374361164bc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sector Defaults" sheetId="6" r:id="Rdb2061943fc543b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Defaults" sheetId="7" r:id="R2df486397f644052"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Control" sheetId="8" r:id="R0f3c982a9aeb4fcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="9" r:id="Ra824b42886aa4070"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="10" r:id="R3ac9938b06514168"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -290,8 +290,8 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="18.5" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="64.62999725341797" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="80.12999725341797" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -325,7 +325,7 @@
         <x:v>Step 2</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Import config/templates/vba/ConfigBuilder.bas into the VBA editor.</x:v>
+        <x:v>Import ConfigBuilder.bas, frmChartWizard.frm, and frmDataSourceWizard.frm from config/templates/vba/.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -333,7 +333,7 @@
         <x:v>Step 3</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Run InstallBuilderButtons once, or run BuildRConfig directly from Excel macros.</x:v>
+        <x:v>Run InstallBuilderButtons once.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -341,7 +341,7 @@
         <x:v>Step 4</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Edit Release Setup, Charts, Data Sources, Sector Defaults, and Chart Defaults.</x:v>
+        <x:v>Click Add Data Source to register Excel sheets or R data functions.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -349,7 +349,7 @@
         <x:v>Step 5</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Click Build R Config to populate the technical config sheets.</x:v>
+        <x:v>Click Add Chart to select sector, data source, fields, labels, forecast settings, and palette settings.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -357,43 +357,59 @@
         <x:v>Step 6</x:v>
       </x:c>
       <x:c r="B9" t="str">
+        <x:v>Click Build R Config to populate the technical config sheets.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>Step 7</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
         <x:v>Click Export Chart Config to create config/releases/&lt;year&gt;/&lt;round&gt;/chart_config.xlsx.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10"/>
-      <x:c r="B10"/>
-    </x:row>
     <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>Macro</x:v>
-      </x:c>
-      <x:c r="B11" t="str">
-        <x:v>What it does</x:v>
-      </x:c>
+      <x:c r="A11"/>
+      <x:c r="B11"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>InstallBuilderButtons</x:v>
+        <x:v>Macro</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Adds clickable buttons to this sheet.</x:v>
+        <x:v>What it does</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>BuildRConfig</x:v>
+        <x:v>InstallBuilderButtons</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>Builds technical config sheets in this workbook.</x:v>
+        <x:v>Adds clickable buttons to this sheet.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>ExportChartConfigXlsx</x:v>
+        <x:v>ShowDataSourceWizard</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>Exports the technical sheets to a macro-free chart_config.xlsx.</x:v>
+        <x:v>Opens the Add Data Source form.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>ShowChartWizard</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>Opens the Add Chart form.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>BuildRConfig / ExportChartConfigXlsx</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Builds and exports the technical R config workbook.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>